<commit_message>
Updating RPA to move to prod env.
</commit_message>
<xml_diff>
--- a/Data/Input/Notifications.xlsx
+++ b/Data/Input/Notifications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SYS-QAUPBOT2\.nuget\packages\scenario4and6.performer\15.0.0\lib\net45\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B9523C3-F0A3-4835-BA47-FA18BC7BE977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB0CB72-5B44-45E2-BF36-FB0148F440C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="26010" windowHeight="20160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
   <si>
     <t>NotificationID</t>
   </si>
@@ -194,10 +194,16 @@
 Thank you</t>
   </si>
   <si>
-    <t>DL-UiPathRPASupport@ralphlauren.com;jose.ordonez@uipath.com</t>
-  </si>
-  <si>
-    <t>Carmen.Suarez@RalphLauren.com;Isabelle.Souksawath@RalphLauren.com;Paula.Pinto@RalphLauren.com;jose.ordonez@uipath.com</t>
+    <t>DL-UiPathRPASupport@ralphlauren.com;jose.ordonez@ralphlauren.com</t>
+  </si>
+  <si>
+    <t>Carmen.Suarez@RalphLauren.com;Isabelle.Souksawath@RalphLauren.com;Paula.Pinto@RalphLauren.com;jose.ordonez@ralphlauren.com</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>jose.ordonez@ralphlauren.com</t>
   </si>
 </sst>
 </file>
@@ -247,7 +253,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -270,12 +276,60 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
@@ -302,19 +356,51 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
     <dxf>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
@@ -474,15 +560,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:F3" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="A1:F3" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="NotificationID" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="NotificationTo" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="NotificationCC" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="NotificationSubject" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="NotificationBody" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{CAB9C0EA-8876-48DE-A84E-4D3352C1A239}" name="Note" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:G3" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:G3" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="NotificationID" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="NotificationTo" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="NotificationCC" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="NotificationSubject" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="NotificationBody" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{CAB9C0EA-8876-48DE-A84E-4D3352C1A239}" name="Note" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{77A6ADA5-55EB-481D-9DD9-1D454F6DF0DC}" name="Column1" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -755,7 +842,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" style="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" style="17" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="94" style="1" customWidth="1"/>
@@ -781,12 +868,15 @@
       <c r="F1" s="5" t="s">
         <v>13</v>
       </c>
+      <c r="G1" s="19" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="2" spans="1:7" ht="101.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="20" t="s">
         <v>36</v>
       </c>
       <c r="C2" s="5"/>
@@ -797,12 +887,13 @@
         <v>18</v>
       </c>
       <c r="F2" s="5"/>
+      <c r="G2" s="18"/>
     </row>
     <row r="3" spans="1:7" ht="116.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="20" t="s">
         <v>36</v>
       </c>
       <c r="C3" s="5"/>
@@ -813,13 +904,14 @@
         <v>17</v>
       </c>
       <c r="F3" s="5"/>
+      <c r="G3" s="21"/>
     </row>
     <row r="4" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="17" t="s">
-        <v>36</v>
+      <c r="B4" s="22" t="s">
+        <v>39</v>
       </c>
       <c r="C4" s="14"/>
       <c r="D4" s="6" t="s">
@@ -829,13 +921,14 @@
         <v>28</v>
       </c>
       <c r="F4" s="5"/>
+      <c r="G4" s="20"/>
     </row>
     <row r="5" spans="1:7" ht="120" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="17" t="s">
-        <v>36</v>
+      <c r="B5" s="22" t="s">
+        <v>39</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="8" t="s">
@@ -845,12 +938,13 @@
         <v>28</v>
       </c>
       <c r="F5" s="5"/>
+      <c r="G5" s="20"/>
     </row>
     <row r="6" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="20" t="s">
         <v>36</v>
       </c>
       <c r="C6" s="12"/>
@@ -861,12 +955,13 @@
         <v>35</v>
       </c>
       <c r="F6" s="5"/>
+      <c r="G6" s="20"/>
     </row>
     <row r="7" spans="1:7" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="20" t="s">
         <v>36</v>
       </c>
       <c r="C7" s="10"/>
@@ -877,12 +972,13 @@
         <v>26</v>
       </c>
       <c r="F7" s="5"/>
+      <c r="G7" s="20"/>
     </row>
     <row r="8" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="16" t="s">
         <v>37</v>
       </c>
       <c r="C8" s="12"/>
@@ -893,6 +989,7 @@
         <v>27</v>
       </c>
       <c r="F8" s="5"/>
+      <c r="G8" s="16"/>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
@@ -930,7 +1027,7 @@
       <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="16" t="s">
         <v>37</v>
       </c>
       <c r="C11" s="15"/>
@@ -946,7 +1043,7 @@
       <c r="G11" s="16"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="17"/>
+      <c r="B12" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updating Login Netweaqver workflow
</commit_message>
<xml_diff>
--- a/Data/Input/Notifications.xlsx
+++ b/Data/Input/Notifications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SYS-QAUPBOT2\.nuget\packages\scenario4and6.performer\15.0.0\lib\net45\Data\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB0CB72-5B44-45E2-BF36-FB0148F440C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB9A43A3-BABF-475E-BC9F-011FDB29E8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="26010" windowHeight="20160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>NotificationID</t>
   </si>
@@ -201,9 +201,6 @@
   </si>
   <si>
     <t>Column1</t>
-  </si>
-  <si>
-    <t>jose.ordonez@ralphlauren.com</t>
   </si>
 </sst>
 </file>
@@ -329,7 +326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
@@ -372,7 +369,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -910,8 +906,8 @@
       <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="22" t="s">
-        <v>39</v>
+      <c r="B4" s="20" t="s">
+        <v>36</v>
       </c>
       <c r="C4" s="14"/>
       <c r="D4" s="6" t="s">
@@ -927,8 +923,8 @@
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>39</v>
+      <c r="B5" s="20" t="s">
+        <v>36</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="8" t="s">

</xml_diff>